<commit_message>
feat(hrm): import roster employee numbers without auto-generating blanks
Excel 员工工号 writes when present. Blank create stays empty; blank
update keeps the existing number. Manual create still auto-generates.
</commit_message>
<xml_diff>
--- a/yudao-module-hrm/yudao-module-hrm-server/src/main/resources/excel/文枢花名册导入模板.xlsx
+++ b/yudao-module-hrm/yudao-module-hrm-server/src/main/resources/excel/文枢花名册导入模板.xlsx
@@ -1570,7 +1570,11 @@
           <t>任职部门</t>
         </is>
       </c>
-      <c r="BC2" s="38" t="n"/>
+      <c r="BC2" s="38" t="inlineStr">
+        <is>
+          <t>员工工号</t>
+        </is>
+      </c>
       <c r="BD2" s="38" t="n"/>
     </row>
     <row r="3" ht="20" customFormat="1" customHeight="1" s="3">

</xml_diff>